<commit_message>
Slight edit of the Chesters Chalcidoidea taxonomy file to facilitate conversion to csv format
</commit_message>
<xml_diff>
--- a/source_data/Chesters_Chalcidoidea_taxonomy_updated.xlsx
+++ b/source_data/Chesters_Chalcidoidea_taxonomy_updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{974FB204-76DC-084C-8B2E-B8E3E70B0693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42EDBD24-02B0-FC4A-885B-9EC816957520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1000" yWindow="500" windowWidth="19540" windowHeight="17440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3225,7 +3225,7 @@
     <t>megastigmid_clade</t>
   </si>
   <si>
-    <t>Delete this entry! Spider sequence…</t>
+    <t>Delete this entry! It is likely a spider sequence.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update to taxonomy of chesters chalcidoids
</commit_message>
<xml_diff>
--- a/source_data/Chesters_Chalcidoidea_taxonomy_updated.xlsx
+++ b/source_data/Chesters_Chalcidoidea_taxonomy_updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42EDBD24-02B0-FC4A-885B-9EC816957520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41D32EE2-281B-B348-AABB-8E41CA5925AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1000" yWindow="500" windowWidth="19540" windowHeight="17440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3225,7 +3225,7 @@
     <t>megastigmid_clade</t>
   </si>
   <si>
-    <t>Delete this entry! It is likely a spider sequence.</t>
+    <t>spider sequence</t>
   </si>
 </sst>
 </file>

</xml_diff>